<commit_message>
Feat v1.2.0: Regla de piso por Evento Maximo e integracion de plantilla Excel actualizada
</commit_message>
<xml_diff>
--- a/Plantilla_Carga_Forecasting.xlsx
+++ b/Plantilla_Carga_Forecasting.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT4"/>
+  <dimension ref="A1:AU4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -477,7 +477,7 @@
     <col width="27" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
@@ -513,6 +513,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,182 +567,187 @@
           <t>Multiplo_Empaque</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Evento_Maximo</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>M01</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>M02</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>M03</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>M04</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>M05</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>M06</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>M07</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>M08</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>M09</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>M10</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>M11</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>M13</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>M14</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>M15</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>M16</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
+      <c r="AB1" s="3" t="inlineStr">
         <is>
           <t>M17</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AC1" s="3" t="inlineStr">
         <is>
           <t>M18</t>
         </is>
       </c>
-      <c r="AC1" s="3" t="inlineStr">
+      <c r="AD1" s="3" t="inlineStr">
         <is>
           <t>M19</t>
         </is>
       </c>
-      <c r="AD1" s="3" t="inlineStr">
+      <c r="AE1" s="3" t="inlineStr">
         <is>
           <t>M20</t>
         </is>
       </c>
-      <c r="AE1" s="3" t="inlineStr">
+      <c r="AF1" s="3" t="inlineStr">
         <is>
           <t>M21</t>
         </is>
       </c>
-      <c r="AF1" s="3" t="inlineStr">
+      <c r="AG1" s="3" t="inlineStr">
         <is>
           <t>M22</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AH1" s="3" t="inlineStr">
         <is>
           <t>M23</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
+      <c r="AI1" s="3" t="inlineStr">
         <is>
           <t>M24</t>
         </is>
       </c>
-      <c r="AI1" s="3" t="inlineStr">
+      <c r="AJ1" s="3" t="inlineStr">
         <is>
           <t>M25</t>
         </is>
       </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="AK1" s="3" t="inlineStr">
         <is>
           <t>M26</t>
         </is>
       </c>
-      <c r="AK1" s="3" t="inlineStr">
+      <c r="AL1" s="3" t="inlineStr">
         <is>
           <t>M27</t>
         </is>
       </c>
-      <c r="AL1" s="3" t="inlineStr">
+      <c r="AM1" s="3" t="inlineStr">
         <is>
           <t>M28</t>
         </is>
       </c>
-      <c r="AM1" s="3" t="inlineStr">
+      <c r="AN1" s="3" t="inlineStr">
         <is>
           <t>M29</t>
         </is>
       </c>
-      <c r="AN1" s="3" t="inlineStr">
+      <c r="AO1" s="3" t="inlineStr">
         <is>
           <t>M30</t>
         </is>
       </c>
-      <c r="AO1" s="3" t="inlineStr">
+      <c r="AP1" s="3" t="inlineStr">
         <is>
           <t>M31</t>
         </is>
       </c>
-      <c r="AP1" s="3" t="inlineStr">
+      <c r="AQ1" s="3" t="inlineStr">
         <is>
           <t>M32</t>
         </is>
       </c>
-      <c r="AQ1" s="3" t="inlineStr">
+      <c r="AR1" s="3" t="inlineStr">
         <is>
           <t>M33</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="AS1" s="3" t="inlineStr">
         <is>
           <t>M34</t>
         </is>
       </c>
-      <c r="AS1" s="3" t="inlineStr">
+      <c r="AT1" s="3" t="inlineStr">
         <is>
           <t>M35</t>
         </is>
       </c>
-      <c r="AT1" s="3" t="inlineStr">
+      <c r="AU1" s="3" t="inlineStr">
         <is>
           <t>M36</t>
         </is>
@@ -781,7 +787,7 @@
         <v>50</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="L2" s="4" t="n">
         <v>0</v>
@@ -796,96 +802,99 @@
         <v>0</v>
       </c>
       <c r="P2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="4" t="n">
         <v>241</v>
       </c>
-      <c r="Q2" s="4" t="n">
+      <c r="R2" s="4" t="n">
         <v>322</v>
       </c>
-      <c r="R2" s="4" t="n">
+      <c r="S2" s="4" t="n">
         <v>296</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="T2" s="4" t="n">
         <v>246</v>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="U2" s="4" t="n">
         <v>339</v>
       </c>
-      <c r="U2" s="4" t="n">
+      <c r="V2" s="4" t="n">
         <v>390</v>
       </c>
-      <c r="V2" s="4" t="n">
+      <c r="W2" s="4" t="n">
         <v>225</v>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="X2" s="4" t="n">
         <v>794</v>
       </c>
-      <c r="X2" s="4" t="n">
+      <c r="Y2" s="4" t="n">
         <v>297</v>
       </c>
-      <c r="Y2" s="4" t="n">
+      <c r="Z2" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="Z2" s="4" t="n">
+      <c r="AA2" s="4" t="n">
         <v>422</v>
       </c>
-      <c r="AA2" s="4" t="n">
+      <c r="AB2" s="4" t="n">
         <v>212</v>
       </c>
-      <c r="AB2" s="4" t="n">
+      <c r="AC2" s="4" t="n">
         <v>274</v>
       </c>
-      <c r="AC2" s="4" t="n">
+      <c r="AD2" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="AD2" s="4" t="n">
+      <c r="AE2" s="4" t="n">
         <v>249</v>
       </c>
-      <c r="AE2" s="4" t="n">
+      <c r="AF2" s="4" t="n">
         <v>271</v>
       </c>
-      <c r="AF2" s="4" t="n">
+      <c r="AG2" s="4" t="n">
         <v>513</v>
       </c>
-      <c r="AG2" s="4" t="n">
+      <c r="AH2" s="4" t="n">
         <v>338</v>
       </c>
-      <c r="AH2" s="4" t="n">
+      <c r="AI2" s="4" t="n">
         <v>343</v>
       </c>
-      <c r="AI2" s="4" t="n">
+      <c r="AJ2" s="4" t="n">
         <v>154</v>
       </c>
-      <c r="AJ2" s="4" t="n">
+      <c r="AK2" s="4" t="n">
         <v>708</v>
       </c>
-      <c r="AK2" s="4" t="n">
+      <c r="AL2" s="4" t="n">
         <v>235</v>
       </c>
-      <c r="AL2" s="4" t="n">
+      <c r="AM2" s="4" t="n">
         <v>310</v>
       </c>
-      <c r="AM2" s="4" t="n">
+      <c r="AN2" s="4" t="n">
         <v>154</v>
       </c>
-      <c r="AN2" s="4" t="n">
+      <c r="AO2" s="4" t="n">
         <v>199</v>
       </c>
-      <c r="AO2" s="4" t="n">
+      <c r="AP2" s="4" t="n">
         <v>205</v>
       </c>
-      <c r="AP2" s="4" t="n">
+      <c r="AQ2" s="4" t="n">
         <v>225</v>
       </c>
-      <c r="AQ2" s="4" t="n">
+      <c r="AR2" s="4" t="n">
         <v>211</v>
       </c>
-      <c r="AR2" s="4" t="n">
+      <c r="AS2" s="4" t="n">
         <v>333</v>
       </c>
-      <c r="AS2" s="4" t="n">
+      <c r="AT2" s="4" t="n">
         <v>342</v>
       </c>
-      <c r="AT2" s="4" t="n">
+      <c r="AU2" s="4" t="n">
         <v>298</v>
       </c>
     </row>
@@ -922,9 +931,7 @@
       <c r="J3" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="K3" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n">
         <v>0</v>
       </c>
@@ -938,96 +945,99 @@
         <v>0</v>
       </c>
       <c r="P3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="4" t="n">
         <v>109</v>
       </c>
-      <c r="Q3" s="4" t="n">
+      <c r="R3" s="4" t="n">
         <v>230</v>
       </c>
-      <c r="R3" s="4" t="n">
+      <c r="S3" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="T3" s="4" t="n">
         <v>141</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="U3" s="4" t="n">
         <v>183</v>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="V3" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="V3" s="4" t="n">
+      <c r="W3" s="4" t="n">
         <v>123</v>
       </c>
-      <c r="W3" s="4" t="n">
+      <c r="X3" s="4" t="n">
         <v>108</v>
       </c>
-      <c r="X3" s="4" t="n">
+      <c r="Y3" s="4" t="n">
         <v>201</v>
       </c>
-      <c r="Y3" s="4" t="n">
+      <c r="Z3" s="4" t="n">
         <v>114</v>
       </c>
-      <c r="Z3" s="4" t="n">
+      <c r="AA3" s="4" t="n">
         <v>168</v>
       </c>
-      <c r="AA3" s="4" t="n">
+      <c r="AB3" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="AB3" s="4" t="n">
+      <c r="AC3" s="4" t="n">
         <v>167</v>
       </c>
-      <c r="AC3" s="4" t="n">
+      <c r="AD3" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="AD3" s="4" t="n">
+      <c r="AE3" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="AE3" s="4" t="n">
+      <c r="AF3" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="AF3" s="4" t="n">
+      <c r="AG3" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="AG3" s="4" t="n">
+      <c r="AH3" s="4" t="n">
         <v>104</v>
       </c>
-      <c r="AH3" s="4" t="n">
+      <c r="AI3" s="4" t="n">
         <v>132</v>
       </c>
-      <c r="AI3" s="4" t="n">
+      <c r="AJ3" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="AJ3" s="4" t="n">
+      <c r="AK3" s="4" t="n">
         <v>82</v>
       </c>
-      <c r="AK3" s="4" t="n">
+      <c r="AL3" s="4" t="n">
         <v>156</v>
       </c>
-      <c r="AL3" s="4" t="n">
+      <c r="AM3" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="AM3" s="4" t="n">
+      <c r="AN3" s="4" t="n">
         <v>116</v>
       </c>
-      <c r="AN3" s="4" t="n">
+      <c r="AO3" s="4" t="n">
         <v>109</v>
       </c>
-      <c r="AO3" s="4" t="n">
+      <c r="AP3" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="AP3" s="4" t="n">
+      <c r="AQ3" s="4" t="n">
         <v>123</v>
       </c>
-      <c r="AQ3" s="4" t="n">
+      <c r="AR3" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="AR3" s="4" t="n">
+      <c r="AS3" s="4" t="n">
         <v>196</v>
       </c>
-      <c r="AS3" s="4" t="n">
+      <c r="AT3" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="AT3" s="4" t="n">
+      <c r="AU3" s="4" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1058,9 +1068,7 @@
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="n">
         <v>0</v>
       </c>
@@ -1074,96 +1082,99 @@
         <v>0</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="V4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="V4" s="4" t="n">
+      <c r="W4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="W4" s="4" t="n">
+      <c r="X4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="X4" s="4" t="n">
+      <c r="Y4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="Y4" s="4" t="n">
+      <c r="Z4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Z4" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="AA4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AB4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="AC4" s="4" t="n">
+      <c r="AD4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="AD4" s="4" t="n">
+      <c r="AE4" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="AE4" s="4" t="n">
+      <c r="AF4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="AF4" s="4" t="n">
+      <c r="AG4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AG4" s="4" t="n">
+      <c r="AH4" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="AH4" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="AI4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AK4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="AL4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="AM4" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="AN4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="AO4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="AQ4" s="4" t="n">
+      <c r="AR4" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="AR4" s="4" t="n">
+      <c r="AS4" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="AS4" s="4" t="n">
+      <c r="AT4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="AT4" s="4" t="n">
+      <c r="AU4" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1178,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1376,15 +1387,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Evento_Maximo</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mayor venta en una exhibición últimos 12 meses. Si Z es 1.65 o 2.05, fija el piso del PDR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>M01 a M36</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Obligatorio</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Historial consecutivo de ventas de los últimos 36 periodos (del más antiguo al más reciente).</t>
         </is>

</xml_diff>

<commit_message>
Feat v1.3.5: Integracion completa de app.py con plantilla oficial de openpyxl y candados dinámicos por SLA
</commit_message>
<xml_diff>
--- a/Plantilla_Carga_Forecasting.xlsx
+++ b/Plantilla_Carga_Forecasting.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU4"/>
+  <dimension ref="A1:AW4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -473,13 +473,13 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
@@ -514,6 +514,8 @@
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
     <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -549,205 +551,215 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>Stock_Maximo_Actual</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>PDR_Actual</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
           <t>Costo_Unitario</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Tasa_Mantenimiento_Anual</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Costo_Ordenar</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Multiplo_Empaque</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Evento_Maximo</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>M01</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>M02</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>M03</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>M04</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>M05</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>M06</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>M07</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>M08</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>M09</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>M10</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>M11</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>M13</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>M14</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="AB1" s="3" t="inlineStr">
         <is>
           <t>M15</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
+      <c r="AC1" s="3" t="inlineStr">
         <is>
           <t>M16</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AD1" s="3" t="inlineStr">
         <is>
           <t>M17</t>
         </is>
       </c>
-      <c r="AC1" s="3" t="inlineStr">
+      <c r="AE1" s="3" t="inlineStr">
         <is>
           <t>M18</t>
         </is>
       </c>
-      <c r="AD1" s="3" t="inlineStr">
+      <c r="AF1" s="3" t="inlineStr">
         <is>
           <t>M19</t>
         </is>
       </c>
-      <c r="AE1" s="3" t="inlineStr">
+      <c r="AG1" s="3" t="inlineStr">
         <is>
           <t>M20</t>
         </is>
       </c>
-      <c r="AF1" s="3" t="inlineStr">
+      <c r="AH1" s="3" t="inlineStr">
         <is>
           <t>M21</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AI1" s="3" t="inlineStr">
         <is>
           <t>M22</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
+      <c r="AJ1" s="3" t="inlineStr">
         <is>
           <t>M23</t>
         </is>
       </c>
-      <c r="AI1" s="3" t="inlineStr">
+      <c r="AK1" s="3" t="inlineStr">
         <is>
           <t>M24</t>
         </is>
       </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="AL1" s="3" t="inlineStr">
         <is>
           <t>M25</t>
         </is>
       </c>
-      <c r="AK1" s="3" t="inlineStr">
+      <c r="AM1" s="3" t="inlineStr">
         <is>
           <t>M26</t>
         </is>
       </c>
-      <c r="AL1" s="3" t="inlineStr">
+      <c r="AN1" s="3" t="inlineStr">
         <is>
           <t>M27</t>
         </is>
       </c>
-      <c r="AM1" s="3" t="inlineStr">
+      <c r="AO1" s="3" t="inlineStr">
         <is>
           <t>M28</t>
         </is>
       </c>
-      <c r="AN1" s="3" t="inlineStr">
+      <c r="AP1" s="3" t="inlineStr">
         <is>
           <t>M29</t>
         </is>
       </c>
-      <c r="AO1" s="3" t="inlineStr">
+      <c r="AQ1" s="3" t="inlineStr">
         <is>
           <t>M30</t>
         </is>
       </c>
-      <c r="AP1" s="3" t="inlineStr">
+      <c r="AR1" s="3" t="inlineStr">
         <is>
           <t>M31</t>
         </is>
       </c>
-      <c r="AQ1" s="3" t="inlineStr">
+      <c r="AS1" s="3" t="inlineStr">
         <is>
           <t>M32</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="AT1" s="3" t="inlineStr">
         <is>
           <t>M33</t>
         </is>
       </c>
-      <c r="AS1" s="3" t="inlineStr">
+      <c r="AU1" s="3" t="inlineStr">
         <is>
           <t>M34</t>
         </is>
       </c>
-      <c r="AT1" s="3" t="inlineStr">
+      <c r="AV1" s="3" t="inlineStr">
         <is>
           <t>M35</t>
         </is>
       </c>
-      <c r="AU1" s="3" t="inlineStr">
+      <c r="AW1" s="3" t="inlineStr">
         <is>
           <t>M36</t>
         </is>
@@ -775,26 +787,26 @@
         <v>12</v>
       </c>
       <c r="G2" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="I2" s="4" t="n">
         <v>6.1</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>0.1</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>450</v>
       </c>
-      <c r="L2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="N2" s="4" t="n">
         <v>0</v>
       </c>
@@ -805,96 +817,102 @@
         <v>0</v>
       </c>
       <c r="Q2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="4" t="n">
         <v>241</v>
       </c>
-      <c r="R2" s="4" t="n">
+      <c r="T2" s="4" t="n">
         <v>322</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="U2" s="4" t="n">
         <v>296</v>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="V2" s="4" t="n">
         <v>246</v>
       </c>
-      <c r="U2" s="4" t="n">
+      <c r="W2" s="4" t="n">
         <v>339</v>
       </c>
-      <c r="V2" s="4" t="n">
+      <c r="X2" s="4" t="n">
         <v>390</v>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="Y2" s="4" t="n">
         <v>225</v>
       </c>
-      <c r="X2" s="4" t="n">
+      <c r="Z2" s="4" t="n">
         <v>794</v>
       </c>
-      <c r="Y2" s="4" t="n">
+      <c r="AA2" s="4" t="n">
         <v>297</v>
       </c>
-      <c r="Z2" s="4" t="n">
+      <c r="AB2" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="AA2" s="4" t="n">
+      <c r="AC2" s="4" t="n">
         <v>422</v>
       </c>
-      <c r="AB2" s="4" t="n">
+      <c r="AD2" s="4" t="n">
         <v>212</v>
       </c>
-      <c r="AC2" s="4" t="n">
+      <c r="AE2" s="4" t="n">
         <v>274</v>
       </c>
-      <c r="AD2" s="4" t="n">
+      <c r="AF2" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="AE2" s="4" t="n">
+      <c r="AG2" s="4" t="n">
         <v>249</v>
       </c>
-      <c r="AF2" s="4" t="n">
+      <c r="AH2" s="4" t="n">
         <v>271</v>
       </c>
-      <c r="AG2" s="4" t="n">
+      <c r="AI2" s="4" t="n">
         <v>513</v>
       </c>
-      <c r="AH2" s="4" t="n">
+      <c r="AJ2" s="4" t="n">
         <v>338</v>
       </c>
-      <c r="AI2" s="4" t="n">
+      <c r="AK2" s="4" t="n">
         <v>343</v>
       </c>
-      <c r="AJ2" s="4" t="n">
+      <c r="AL2" s="4" t="n">
         <v>154</v>
       </c>
-      <c r="AK2" s="4" t="n">
+      <c r="AM2" s="4" t="n">
         <v>708</v>
       </c>
-      <c r="AL2" s="4" t="n">
+      <c r="AN2" s="4" t="n">
         <v>235</v>
       </c>
-      <c r="AM2" s="4" t="n">
+      <c r="AO2" s="4" t="n">
         <v>310</v>
       </c>
-      <c r="AN2" s="4" t="n">
+      <c r="AP2" s="4" t="n">
         <v>154</v>
       </c>
-      <c r="AO2" s="4" t="n">
+      <c r="AQ2" s="4" t="n">
         <v>199</v>
       </c>
-      <c r="AP2" s="4" t="n">
+      <c r="AR2" s="4" t="n">
         <v>205</v>
       </c>
-      <c r="AQ2" s="4" t="n">
+      <c r="AS2" s="4" t="n">
         <v>225</v>
       </c>
-      <c r="AR2" s="4" t="n">
+      <c r="AT2" s="4" t="n">
         <v>211</v>
       </c>
-      <c r="AS2" s="4" t="n">
+      <c r="AU2" s="4" t="n">
         <v>333</v>
       </c>
-      <c r="AT2" s="4" t="n">
+      <c r="AV2" s="4" t="n">
         <v>342</v>
       </c>
-      <c r="AU2" s="4" t="n">
+      <c r="AW2" s="4" t="n">
         <v>298</v>
       </c>
     </row>
@@ -920,24 +938,24 @@
         <v>5</v>
       </c>
       <c r="G3" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="I3" s="4" t="n">
         <v>6.16</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>0.1</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="M3" s="4" t="n"/>
       <c r="N3" s="4" t="n">
         <v>0</v>
       </c>
@@ -948,96 +966,102 @@
         <v>0</v>
       </c>
       <c r="Q3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="4" t="n">
         <v>109</v>
       </c>
-      <c r="R3" s="4" t="n">
+      <c r="T3" s="4" t="n">
         <v>230</v>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="U3" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="V3" s="4" t="n">
         <v>141</v>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="W3" s="4" t="n">
         <v>183</v>
       </c>
-      <c r="V3" s="4" t="n">
+      <c r="X3" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="W3" s="4" t="n">
+      <c r="Y3" s="4" t="n">
         <v>123</v>
       </c>
-      <c r="X3" s="4" t="n">
+      <c r="Z3" s="4" t="n">
         <v>108</v>
       </c>
-      <c r="Y3" s="4" t="n">
+      <c r="AA3" s="4" t="n">
         <v>201</v>
       </c>
-      <c r="Z3" s="4" t="n">
+      <c r="AB3" s="4" t="n">
         <v>114</v>
       </c>
-      <c r="AA3" s="4" t="n">
+      <c r="AC3" s="4" t="n">
         <v>168</v>
       </c>
-      <c r="AB3" s="4" t="n">
+      <c r="AD3" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="AC3" s="4" t="n">
+      <c r="AE3" s="4" t="n">
         <v>167</v>
       </c>
-      <c r="AD3" s="4" t="n">
+      <c r="AF3" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="AE3" s="4" t="n">
+      <c r="AG3" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="AF3" s="4" t="n">
+      <c r="AH3" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="AG3" s="4" t="n">
+      <c r="AI3" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="AH3" s="4" t="n">
+      <c r="AJ3" s="4" t="n">
         <v>104</v>
       </c>
-      <c r="AI3" s="4" t="n">
+      <c r="AK3" s="4" t="n">
         <v>132</v>
       </c>
-      <c r="AJ3" s="4" t="n">
+      <c r="AL3" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="AK3" s="4" t="n">
+      <c r="AM3" s="4" t="n">
         <v>82</v>
       </c>
-      <c r="AL3" s="4" t="n">
+      <c r="AN3" s="4" t="n">
         <v>156</v>
       </c>
-      <c r="AM3" s="4" t="n">
+      <c r="AO3" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="AN3" s="4" t="n">
+      <c r="AP3" s="4" t="n">
         <v>116</v>
       </c>
-      <c r="AO3" s="4" t="n">
+      <c r="AQ3" s="4" t="n">
         <v>109</v>
       </c>
-      <c r="AP3" s="4" t="n">
+      <c r="AR3" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="AQ3" s="4" t="n">
+      <c r="AS3" s="4" t="n">
         <v>123</v>
       </c>
-      <c r="AR3" s="4" t="n">
+      <c r="AT3" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="AS3" s="4" t="n">
+      <c r="AU3" s="4" t="n">
         <v>196</v>
       </c>
-      <c r="AT3" s="4" t="n">
+      <c r="AV3" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="AU3" s="4" t="n">
+      <c r="AW3" s="4" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1063,18 +1087,18 @@
         <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>2.5</v>
       </c>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
       <c r="N4" s="4" t="n">
         <v>0</v>
       </c>
@@ -1085,96 +1109,102 @@
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="V4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="W4" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="V4" s="4" t="n">
+      <c r="X4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="W4" s="4" t="n">
+      <c r="Y4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="X4" s="4" t="n">
+      <c r="Z4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="Y4" s="4" t="n">
+      <c r="AA4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="Z4" s="4" t="n">
+      <c r="AB4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="AA4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="AC4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="AD4" s="4" t="n">
+      <c r="AF4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="AE4" s="4" t="n">
+      <c r="AG4" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="AF4" s="4" t="n">
+      <c r="AH4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="AG4" s="4" t="n">
+      <c r="AI4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH4" s="4" t="n">
+      <c r="AJ4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="AI4" s="4" t="n">
+      <c r="AK4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="AJ4" s="4" t="n">
+      <c r="AL4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="AK4" s="4" t="n">
+      <c r="AM4" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="AL4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM4" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="AN4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="AO4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AP4" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="AQ4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="AR4" s="4" t="n">
+      <c r="AT4" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="AS4" s="4" t="n">
+      <c r="AU4" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="AT4" s="4" t="n">
+      <c r="AV4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="AU4" s="4" t="n">
+      <c r="AW4" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1189,12 +1219,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="97" customWidth="1" min="3" max="3"/>
+    <col width="145" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1295,7 +1325,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Coeficiente Z deseado (1.65 = 95%, 2.05 = 98%, 1.28 = 90%).</t>
+          <t>Coeficiente Z deseado (1.65 = 95%, 2.05 = 98%, 1.28 = 90%, 1.04 = 85%).</t>
         </is>
       </c>
     </row>
@@ -1312,14 +1342,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Stock disponible. Si se llena, calcula la sugerencia de reabasto neto.</t>
+          <t>Stock disponible en sistema (ERP). Si se llena, calcula el reabasto sugerido neto.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Costo_Unitario</t>
+          <t>Stock_Maximo_Actual</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1329,14 +1359,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Costo de compra unitario. Requerido si se calculará Lote Económico (Q*).</t>
+          <t>Stock Máximo parametrizado actualmente en el ERP. Usado para auditar reducciones drásticas (&gt;200% en Z alta prioridad o &gt;500% en Z estándar).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tasa_Mantenimiento_Anual</t>
+          <t>PDR_Actual</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1346,14 +1376,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Porcentaje decimal (ej. 0.10). Si no se entrega junto con Costo_Ordenar, se omite Q*.</t>
+          <t>Punto de Reorden parametrizado actualmente en el ERP.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Costo_Ordenar</t>
+          <t>Costo_Unitario</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1363,14 +1393,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Costo por emisión de orden. Si no se entrega junto con Tasa, se omite Q*.</t>
+          <t>Costo de compra unitario. Requerido si se calculará Lote Económico (Q*).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Multiplo_Empaque</t>
+          <t>Tasa_Mantenimiento_Anual</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1380,14 +1410,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lote o tamaño de caja. Si se omite, los stocks no se redondean a múltiplos.</t>
+          <t>Porcentaje decimal (ej. 0.10). Si no se entrega junto con Costo_Ordenar, se omite Q*.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Evento_Maximo</t>
+          <t>Costo_Ordenar</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1397,22 +1427,56 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mayor venta en una exhibición últimos 12 meses. Si Z es 1.65 o 2.05, fija el piso del PDR.</t>
+          <t>Costo por emisión de orden. Si no se entrega junto con Tasa, se omite Q*.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Multiplo_Empaque</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lote o tamaño de caja. Si se omite, los stocks no se redondean a múltiplos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Evento_Maximo</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mayor venta en una exhibición últimos 12 meses. Si Z es 1.65 o 2.05, fija el piso del PDR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>M01 a M36</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Obligatorio</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Historial consecutivo de ventas de los últimos 36 periodos (del más antiguo al más reciente).</t>
         </is>

</xml_diff>